<commit_message>
Update daily stock screen
</commit_message>
<xml_diff>
--- a/output/daily_screen_20260911.xlsx
+++ b/output/daily_screen_20260911.xlsx
@@ -662,24 +662,24 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>73.59999999999999</v>
+        <v>63.8</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Heavy Sell</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>20260911</t>
+          <t>20260914</t>
         </is>
       </c>
       <c r="H2" t="n">
-        <v>700000</v>
+        <v>485000</v>
       </c>
       <c r="I2" t="inlineStr"/>
       <c r="J2" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="K2" t="b">
         <v>0</v>
@@ -691,10 +691,10 @@
         <v>700000</v>
       </c>
       <c r="N2" t="n">
-        <v>0</v>
+        <v>-215000</v>
       </c>
       <c r="O2" t="n">
-        <v>0</v>
+        <v>-0.3071428571428572</v>
       </c>
       <c r="P2" t="n">
         <v>1330</v>
@@ -703,7 +703,7 @@
         <v>1330</v>
       </c>
       <c r="R2" t="n">
-        <v>5050252</v>
+        <v>4943644</v>
       </c>
       <c r="S2" t="n">
         <v>1288</v>
@@ -721,13 +721,13 @@
         <v>39.90773424780309</v>
       </c>
       <c r="X2" t="n">
-        <v>32.83570320214118</v>
+        <v>32.8357032021411</v>
       </c>
       <c r="Y2" t="n">
-        <v>7.072031045661916</v>
+        <v>7.072031045661994</v>
       </c>
       <c r="Z2" t="n">
-        <v>5.684694423661924</v>
+        <v>5.684694423662027</v>
       </c>
       <c r="AA2" t="b">
         <v>1</v>
@@ -804,20 +804,20 @@
         </is>
       </c>
       <c r="E3" t="n">
-        <v>59</v>
+        <v>68.40000000000001</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Heavy Buy</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>20260911</t>
+          <t>20260914</t>
         </is>
       </c>
       <c r="H3" t="n">
-        <v>2477000</v>
+        <v>2512000</v>
       </c>
       <c r="I3" t="inlineStr"/>
       <c r="J3" t="n">
@@ -833,10 +833,10 @@
         <v>2477000</v>
       </c>
       <c r="N3" t="n">
-        <v>0</v>
+        <v>35000</v>
       </c>
       <c r="O3" t="n">
-        <v>0</v>
+        <v>0.0141299959628583</v>
       </c>
       <c r="P3" t="n">
         <v>5765</v>
@@ -845,7 +845,7 @@
         <v>5765</v>
       </c>
       <c r="R3" t="n">
-        <v>707334</v>
+        <v>671341</v>
       </c>
       <c r="S3" t="n">
         <v>5704</v>
@@ -944,20 +944,20 @@
         </is>
       </c>
       <c r="E4" t="n">
-        <v>54.40000000000001</v>
+        <v>64.2</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Heavy Buy</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>20260911</t>
+          <t>20260914</t>
         </is>
       </c>
       <c r="H4" t="n">
-        <v>372000</v>
+        <v>413000</v>
       </c>
       <c r="I4" t="inlineStr"/>
       <c r="J4" t="n">
@@ -973,10 +973,10 @@
         <v>372000</v>
       </c>
       <c r="N4" t="n">
-        <v>0</v>
+        <v>41000</v>
       </c>
       <c r="O4" t="n">
-        <v>0</v>
+        <v>0.1102150537634409</v>
       </c>
       <c r="P4" t="n">
         <v>6120</v>
@@ -985,7 +985,7 @@
         <v>6120</v>
       </c>
       <c r="R4" t="n">
-        <v>1476663</v>
+        <v>1425347</v>
       </c>
       <c r="S4" t="n">
         <v>6033</v>
@@ -1093,7 +1093,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>20260911</t>
+          <t>20260914</t>
         </is>
       </c>
       <c r="H5" t="n">
@@ -1125,7 +1125,7 @@
         <v>140.5</v>
       </c>
       <c r="R5" t="n">
-        <v>120621193</v>
+        <v>119260816</v>
       </c>
       <c r="S5" t="n">
         <v>140.9</v>
@@ -1140,16 +1140,16 @@
         <v>137.1627202351888</v>
       </c>
       <c r="W5" t="n">
-        <v>4.690909053504299</v>
+        <v>4.690909053504328</v>
       </c>
       <c r="X5" t="n">
-        <v>2.962828799205447</v>
+        <v>2.962828799205475</v>
       </c>
       <c r="Y5" t="n">
-        <v>1.728080254298852</v>
+        <v>1.728080254298853</v>
       </c>
       <c r="Z5" t="n">
-        <v>2.167341712366061</v>
+        <v>2.167341712366063</v>
       </c>
       <c r="AA5" t="b">
         <v>0</v>
@@ -1235,7 +1235,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>20260911</t>
+          <t>20260914</t>
         </is>
       </c>
       <c r="H6" t="n">
@@ -1267,7 +1267,7 @@
         <v>2310</v>
       </c>
       <c r="R6" t="n">
-        <v>1888918</v>
+        <v>1627022</v>
       </c>
       <c r="S6" t="n">
         <v>2362</v>
@@ -1282,16 +1282,16 @@
         <v>1955.745255533854</v>
       </c>
       <c r="W6" t="n">
-        <v>43.80731406619134</v>
+        <v>43.80731406619088</v>
       </c>
       <c r="X6" t="n">
-        <v>85.59262024075896</v>
+        <v>85.59262024075835</v>
       </c>
       <c r="Y6" t="n">
-        <v>-41.78530617456762</v>
+        <v>-41.78530617456747</v>
       </c>
       <c r="Z6" t="n">
-        <v>-36.142077953157</v>
+        <v>-36.1420779531568</v>
       </c>
       <c r="AA6" t="b">
         <v>0</v>
@@ -1373,7 +1373,7 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>20260911</t>
+          <t>20260914</t>
         </is>
       </c>
       <c r="H7" t="n">
@@ -1405,7 +1405,7 @@
         <v>6660</v>
       </c>
       <c r="R7" t="n">
-        <v>1980286</v>
+        <v>1858248</v>
       </c>
       <c r="S7" t="n">
         <v>6682</v>
@@ -1423,13 +1423,13 @@
         <v>278.6948379755941</v>
       </c>
       <c r="X7" t="n">
-        <v>458.1673203770637</v>
+        <v>458.1673203770636</v>
       </c>
       <c r="Y7" t="n">
-        <v>-179.4724824014697</v>
+        <v>-179.4724824014696</v>
       </c>
       <c r="Z7" t="n">
-        <v>-166.4546906656735</v>
+        <v>-166.4546906656734</v>
       </c>
       <c r="AA7" t="b">
         <v>0</v>
@@ -1511,7 +1511,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>20260911</t>
+          <t>20260914</t>
         </is>
       </c>
       <c r="H8" t="n">
@@ -1543,7 +1543,7 @@
         <v>2150</v>
       </c>
       <c r="R8" t="n">
-        <v>1017797</v>
+        <v>991243</v>
       </c>
       <c r="S8" t="n">
         <v>2211</v>
@@ -1558,16 +1558,16 @@
         <v>1718.324682617188</v>
       </c>
       <c r="W8" t="n">
-        <v>81.72624149239118</v>
+        <v>81.72624149239073</v>
       </c>
       <c r="X8" t="n">
-        <v>107.6367292446171</v>
+        <v>107.6367292446166</v>
       </c>
       <c r="Y8" t="n">
-        <v>-25.91048775222588</v>
+        <v>-25.91048775222589</v>
       </c>
       <c r="Z8" t="n">
-        <v>-16.94700402976784</v>
+        <v>-16.94700402976785</v>
       </c>
       <c r="AA8" t="b">
         <v>0</v>
@@ -1651,7 +1651,7 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>20260911</t>
+          <t>20260914</t>
         </is>
       </c>
       <c r="H9" t="n">
@@ -1683,7 +1683,7 @@
         <v>101</v>
       </c>
       <c r="R9" t="n">
-        <v>6774857</v>
+        <v>6754463</v>
       </c>
       <c r="S9" t="n">
         <v>99.85999908447266</v>
@@ -1701,13 +1701,13 @@
         <v>2.548482324952374</v>
       </c>
       <c r="X9" t="n">
-        <v>2.541357232987988</v>
+        <v>2.541357232987986</v>
       </c>
       <c r="Y9" t="n">
-        <v>0.007125091964386154</v>
+        <v>0.007125091964388375</v>
       </c>
       <c r="Z9" t="n">
-        <v>0.02675220142829859</v>
+        <v>0.02675220142830126</v>
       </c>
       <c r="AA9" t="b">
         <v>0</v>
@@ -1793,7 +1793,7 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>20260911</t>
+          <t>20260914</t>
         </is>
       </c>
       <c r="H10" t="n">
@@ -1825,7 +1825,7 @@
         <v>263</v>
       </c>
       <c r="R10" t="n">
-        <v>17729240</v>
+        <v>16992490</v>
       </c>
       <c r="S10" t="n">
         <v>269.2</v>
@@ -1843,13 +1843,13 @@
         <v>4.809530175251439</v>
       </c>
       <c r="X10" t="n">
-        <v>4.577638248231361</v>
+        <v>4.577638248231355</v>
       </c>
       <c r="Y10" t="n">
-        <v>0.2318919270200777</v>
+        <v>0.2318919270200839</v>
       </c>
       <c r="Z10" t="n">
-        <v>1.382907551939251</v>
+        <v>1.382907551939258</v>
       </c>
       <c r="AA10" t="b">
         <v>0</v>
@@ -1912,12 +1912,12 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>6510</t>
+          <t>2454</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>精測</t>
+          <t>聯發科</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -1926,7 +1926,7 @@
         </is>
       </c>
       <c r="E11" t="n">
-        <v>44.2</v>
+        <v>43</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
@@ -1935,15 +1935,15 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>20260911</t>
+          <t>20260914</t>
         </is>
       </c>
       <c r="H11" t="n">
-        <v>637000</v>
+        <v>5186000</v>
       </c>
       <c r="I11" t="inlineStr"/>
       <c r="J11" t="n">
-        <v>28</v>
+        <v>13</v>
       </c>
       <c r="K11" t="b">
         <v>0</v>
@@ -1952,7 +1952,7 @@
         <v>0</v>
       </c>
       <c r="M11" t="n">
-        <v>637000</v>
+        <v>5186000</v>
       </c>
       <c r="N11" t="n">
         <v>0</v>
@@ -1961,61 +1961,61 @@
         <v>0</v>
       </c>
       <c r="P11" t="n">
-        <v>3480</v>
+        <v>4585</v>
       </c>
       <c r="Q11" t="n">
-        <v>3480</v>
+        <v>4585</v>
       </c>
       <c r="R11" t="n">
-        <v>1104551</v>
+        <v>6841032</v>
       </c>
       <c r="S11" t="n">
-        <v>3570</v>
+        <v>4680</v>
       </c>
       <c r="T11" t="n">
-        <v>3052</v>
+        <v>4161.75</v>
       </c>
       <c r="U11" t="n">
-        <v>3027.5</v>
+        <v>4143</v>
       </c>
       <c r="V11" t="n">
-        <v>2927.079142252604</v>
+        <v>3986.717415364583</v>
       </c>
       <c r="W11" t="n">
-        <v>210.4160916274091</v>
+        <v>197.1743621014048</v>
       </c>
       <c r="X11" t="n">
-        <v>165.3148866757768</v>
+        <v>155.950178214217</v>
       </c>
       <c r="Y11" t="n">
-        <v>45.1012049516323</v>
+        <v>41.22418388718773</v>
       </c>
       <c r="Z11" t="n">
-        <v>76.13910869752343</v>
+        <v>66.74904199942983</v>
       </c>
       <c r="AA11" t="b">
         <v>0</v>
       </c>
       <c r="AB11" t="n">
-        <v>0.1638795986622072</v>
+        <v>0.0890736342042755</v>
       </c>
       <c r="AC11" t="n">
-        <v>-0.03081196953418652</v>
+        <v>0.05065948181334012</v>
       </c>
       <c r="AD11" t="n">
-        <v>0.1557191186875424</v>
+        <v>0.08091315422961065</v>
       </c>
       <c r="AE11" t="n">
-        <v>-0.03751376606863144</v>
+        <v>0.04395768527889521</v>
       </c>
       <c r="AF11" t="n">
-        <v>0.1932328847561738</v>
+        <v>0.03695546895071544</v>
       </c>
       <c r="AG11" t="n">
-        <v>92</v>
+        <v>82</v>
       </c>
       <c r="AH11" t="n">
-        <v>64</v>
+        <v>82</v>
       </c>
       <c r="AI11" t="b">
         <v>1</v>
@@ -2054,12 +2054,12 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2454</t>
+          <t>3711</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>聯發科</t>
+          <t>日月光投控</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -2068,7 +2068,7 @@
         </is>
       </c>
       <c r="E12" t="n">
-        <v>43</v>
+        <v>42.8</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
@@ -2077,24 +2077,24 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>20260911</t>
+          <t>20260914</t>
         </is>
       </c>
       <c r="H12" t="n">
-        <v>5186000</v>
+        <v>16811000</v>
       </c>
       <c r="I12" t="inlineStr"/>
       <c r="J12" t="n">
-        <v>13</v>
+        <v>4</v>
       </c>
       <c r="K12" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L12" t="b">
         <v>0</v>
       </c>
       <c r="M12" t="n">
-        <v>5186000</v>
+        <v>16811000</v>
       </c>
       <c r="N12" t="n">
         <v>0</v>
@@ -2103,61 +2103,61 @@
         <v>0</v>
       </c>
       <c r="P12" t="n">
-        <v>4585</v>
+        <v>618</v>
       </c>
       <c r="Q12" t="n">
-        <v>4585</v>
+        <v>618</v>
       </c>
       <c r="R12" t="n">
-        <v>7568846</v>
+        <v>21540625</v>
       </c>
       <c r="S12" t="n">
-        <v>4680</v>
+        <v>629.4</v>
       </c>
       <c r="T12" t="n">
-        <v>4161.75</v>
+        <v>604.35</v>
       </c>
       <c r="U12" t="n">
-        <v>4143</v>
+        <v>604.25</v>
       </c>
       <c r="V12" t="n">
-        <v>3986.717415364583</v>
+        <v>621.1943979899089</v>
       </c>
       <c r="W12" t="n">
-        <v>197.1743621014057</v>
+        <v>8.168661987707651</v>
       </c>
       <c r="X12" t="n">
-        <v>155.950178214218</v>
+        <v>3.518014378830946</v>
       </c>
       <c r="Y12" t="n">
-        <v>41.22418388718768</v>
+        <v>4.650647608876705</v>
       </c>
       <c r="Z12" t="n">
-        <v>66.74904199942978</v>
+        <v>7.157082383841484</v>
       </c>
       <c r="AA12" t="b">
         <v>0</v>
       </c>
       <c r="AB12" t="n">
-        <v>0.0890736342042755</v>
+        <v>0.003246753246753276</v>
       </c>
       <c r="AC12" t="n">
-        <v>0.05065948181334012</v>
+        <v>0.01737144639336097</v>
       </c>
       <c r="AD12" t="n">
-        <v>0.08091315422961065</v>
+        <v>-0.004913726727911572</v>
       </c>
       <c r="AE12" t="n">
-        <v>0.04395768527889521</v>
+        <v>0.01066964985891605</v>
       </c>
       <c r="AF12" t="n">
-        <v>0.03695546895071544</v>
+        <v>-0.01558337658682762</v>
       </c>
       <c r="AG12" t="n">
-        <v>82</v>
+        <v>50</v>
       </c>
       <c r="AH12" t="n">
-        <v>82</v>
+        <v>76</v>
       </c>
       <c r="AI12" t="b">
         <v>1</v>
@@ -2196,12 +2196,12 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>3711</t>
+          <t>2330</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>日月光投控</t>
+          <t>台積電</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -2219,15 +2219,15 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>20260911</t>
+          <t>20260914</t>
         </is>
       </c>
       <c r="H13" t="n">
-        <v>16811000</v>
+        <v>11864000</v>
       </c>
       <c r="I13" t="inlineStr"/>
       <c r="J13" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="K13" t="b">
         <v>1</v>
@@ -2236,7 +2236,7 @@
         <v>0</v>
       </c>
       <c r="M13" t="n">
-        <v>16811000</v>
+        <v>11864000</v>
       </c>
       <c r="N13" t="n">
         <v>0</v>
@@ -2245,84 +2245,82 @@
         <v>0</v>
       </c>
       <c r="P13" t="n">
-        <v>618</v>
+        <v>2410</v>
       </c>
       <c r="Q13" t="n">
-        <v>618</v>
+        <v>2410</v>
       </c>
       <c r="R13" t="n">
-        <v>22638149</v>
+        <v>18149016</v>
       </c>
       <c r="S13" t="n">
-        <v>629.4</v>
+        <v>2451</v>
       </c>
       <c r="T13" t="n">
-        <v>604.35</v>
+        <v>2411</v>
       </c>
       <c r="U13" t="n">
-        <v>604.25</v>
+        <v>2410.25</v>
       </c>
       <c r="V13" t="n">
-        <v>621.1943979899089</v>
+        <v>2399.75</v>
       </c>
       <c r="W13" t="n">
-        <v>8.168661987707651</v>
+        <v>12.57621423813816</v>
       </c>
       <c r="X13" t="n">
-        <v>3.518014378830951</v>
+        <v>12.66069475230742</v>
       </c>
       <c r="Y13" t="n">
-        <v>4.650647608876699</v>
+        <v>-0.08448051416925395</v>
       </c>
       <c r="Z13" t="n">
-        <v>7.157082383841478</v>
+        <v>5.141822621183577</v>
       </c>
       <c r="AA13" t="b">
         <v>0</v>
       </c>
       <c r="AB13" t="n">
-        <v>0.003246753246753276</v>
+        <v>0.006263048016701411</v>
       </c>
       <c r="AC13" t="n">
-        <v>0.01737144639336097</v>
+        <v>0</v>
       </c>
       <c r="AD13" t="n">
-        <v>-0.004913726727911572</v>
+        <v>-0.001897431957963436</v>
       </c>
       <c r="AE13" t="n">
-        <v>0.01066964985891605</v>
+        <v>-0.006701796534444915</v>
       </c>
       <c r="AF13" t="n">
-        <v>-0.01558337658682762</v>
+        <v>0.004804364576481479</v>
       </c>
       <c r="AG13" t="n">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="AH13" t="n">
-        <v>76</v>
+        <v>70</v>
       </c>
       <c r="AI13" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AJ13" t="b">
         <v>1</v>
       </c>
       <c r="AK13" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AL13" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AM13" t="b">
         <v>0</v>
       </c>
       <c r="AN13" t="b">
-        <v>0</v>
-      </c>
-      <c r="AO13" t="inlineStr">
-        <is>
-          <t>Already &gt; 0</t>
-        </is>
+        <v>1</v>
+      </c>
+      <c r="AO13" t="n">
+        <v>2414.82</v>
       </c>
       <c r="AP13" t="inlineStr">
         <is>
@@ -2338,12 +2336,12 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2330</t>
+          <t>3017</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>台積電</t>
+          <t>奇鋐</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -2352,7 +2350,7 @@
         </is>
       </c>
       <c r="E14" t="n">
-        <v>42.8</v>
+        <v>41.6</v>
       </c>
       <c r="F14" t="inlineStr">
         <is>
@@ -2361,24 +2359,24 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>20260911</t>
+          <t>20260914</t>
         </is>
       </c>
       <c r="H14" t="n">
-        <v>11864000</v>
+        <v>5949000</v>
       </c>
       <c r="I14" t="inlineStr"/>
       <c r="J14" t="n">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="K14" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L14" t="b">
         <v>0</v>
       </c>
       <c r="M14" t="n">
-        <v>11864000</v>
+        <v>5949000</v>
       </c>
       <c r="N14" t="n">
         <v>0</v>
@@ -2387,64 +2385,64 @@
         <v>0</v>
       </c>
       <c r="P14" t="n">
-        <v>2410</v>
+        <v>3370</v>
       </c>
       <c r="Q14" t="n">
-        <v>2410</v>
+        <v>3370</v>
       </c>
       <c r="R14" t="n">
-        <v>20883341</v>
+        <v>2005532</v>
       </c>
       <c r="S14" t="n">
-        <v>2451</v>
+        <v>3383</v>
       </c>
       <c r="T14" t="n">
-        <v>2411</v>
+        <v>3234.176245117188</v>
       </c>
       <c r="U14" t="n">
-        <v>2410.25</v>
+        <v>3226.472351074219</v>
       </c>
       <c r="V14" t="n">
-        <v>2399.75</v>
+        <v>2723.961385091146</v>
       </c>
       <c r="W14" t="n">
-        <v>12.57621423813634</v>
+        <v>105.335889759589</v>
       </c>
       <c r="X14" t="n">
-        <v>12.66069475230379</v>
+        <v>130.5570063572081</v>
       </c>
       <c r="Y14" t="n">
-        <v>-0.08448051416744384</v>
+        <v>-25.22111659761913</v>
       </c>
       <c r="Z14" t="n">
-        <v>5.141822621185385</v>
+        <v>-18.00179342998683</v>
       </c>
       <c r="AA14" t="b">
         <v>0</v>
       </c>
       <c r="AB14" t="n">
-        <v>0.006263048016701411</v>
+        <v>0.04791094906880033</v>
       </c>
       <c r="AC14" t="n">
-        <v>0</v>
+        <v>0.4124966090818585</v>
       </c>
       <c r="AD14" t="n">
-        <v>-0.001897431957963436</v>
+        <v>0.03975046909413549</v>
       </c>
       <c r="AE14" t="n">
-        <v>-0.006701796534444915</v>
+        <v>0.4057948125474136</v>
       </c>
       <c r="AF14" t="n">
-        <v>0.004804364576481479</v>
+        <v>-0.3660443434532781</v>
       </c>
       <c r="AG14" t="n">
-        <v>52</v>
+        <v>72</v>
       </c>
       <c r="AH14" t="n">
-        <v>70</v>
+        <v>98</v>
       </c>
       <c r="AI14" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AJ14" t="b">
         <v>1</v>
@@ -2462,7 +2460,7 @@
         <v>1</v>
       </c>
       <c r="AO14" t="n">
-        <v>2414.82</v>
+        <v>3659.82</v>
       </c>
       <c r="AP14" t="inlineStr">
         <is>
@@ -2478,12 +2476,12 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>3017</t>
+          <t>6271</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>奇鋐</t>
+          <t>同欣電</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -2492,7 +2490,7 @@
         </is>
       </c>
       <c r="E15" t="n">
-        <v>41.6</v>
+        <v>40.8</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
@@ -2501,15 +2499,15 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>20260911</t>
+          <t>20260914</t>
         </is>
       </c>
       <c r="H15" t="n">
-        <v>5949000</v>
+        <v>2222000</v>
       </c>
       <c r="I15" t="inlineStr"/>
       <c r="J15" t="n">
-        <v>11</v>
+        <v>23</v>
       </c>
       <c r="K15" t="b">
         <v>0</v>
@@ -2518,7 +2516,7 @@
         <v>0</v>
       </c>
       <c r="M15" t="n">
-        <v>5949000</v>
+        <v>2222000</v>
       </c>
       <c r="N15" t="n">
         <v>0</v>
@@ -2527,61 +2525,61 @@
         <v>0</v>
       </c>
       <c r="P15" t="n">
-        <v>3370</v>
+        <v>220</v>
       </c>
       <c r="Q15" t="n">
-        <v>3370</v>
+        <v>220</v>
       </c>
       <c r="R15" t="n">
-        <v>2108980</v>
+        <v>2216922</v>
       </c>
       <c r="S15" t="n">
-        <v>3383</v>
+        <v>225.8</v>
       </c>
       <c r="T15" t="n">
-        <v>3234.176245117188</v>
+        <v>212.425</v>
       </c>
       <c r="U15" t="n">
-        <v>3226.472351074219</v>
+        <v>211.125</v>
       </c>
       <c r="V15" t="n">
-        <v>2723.961385091146</v>
+        <v>216.1166666666667</v>
       </c>
       <c r="W15" t="n">
-        <v>105.335889759589</v>
+        <v>6.068834410018638</v>
       </c>
       <c r="X15" t="n">
-        <v>130.5570063572082</v>
+        <v>6.737541555554651</v>
       </c>
       <c r="Y15" t="n">
-        <v>-25.22111659761919</v>
+        <v>-0.668707145536013</v>
       </c>
       <c r="Z15" t="n">
-        <v>-18.00179342998689</v>
+        <v>0.439375949514023</v>
       </c>
       <c r="AA15" t="b">
         <v>0</v>
       </c>
       <c r="AB15" t="n">
-        <v>0.04791094906880033</v>
+        <v>0.134020618556701</v>
       </c>
       <c r="AC15" t="n">
-        <v>0.4124966090818585</v>
+        <v>-0.09278350515463918</v>
       </c>
       <c r="AD15" t="n">
-        <v>0.03975046909413549</v>
+        <v>0.1258601385820362</v>
       </c>
       <c r="AE15" t="n">
-        <v>0.4057948125474136</v>
+        <v>-0.09948530168908409</v>
       </c>
       <c r="AF15" t="n">
-        <v>-0.3660443434532781</v>
+        <v>0.2253454402711202</v>
       </c>
       <c r="AG15" t="n">
-        <v>72</v>
+        <v>88</v>
       </c>
       <c r="AH15" t="n">
-        <v>98</v>
+        <v>42</v>
       </c>
       <c r="AI15" t="b">
         <v>1</v>
@@ -2602,7 +2600,7 @@
         <v>1</v>
       </c>
       <c r="AO15" t="n">
-        <v>3659.82</v>
+        <v>227.92</v>
       </c>
       <c r="AP15" t="inlineStr">
         <is>
@@ -2618,12 +2616,12 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>6271</t>
+          <t>2481</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>同欣電</t>
+          <t>強茂</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -2632,7 +2630,7 @@
         </is>
       </c>
       <c r="E16" t="n">
-        <v>40.8</v>
+        <v>39.4</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
@@ -2641,15 +2639,15 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>20260911</t>
+          <t>20260914</t>
         </is>
       </c>
       <c r="H16" t="n">
-        <v>2222000</v>
+        <v>5000</v>
       </c>
       <c r="I16" t="inlineStr"/>
       <c r="J16" t="n">
-        <v>23</v>
+        <v>34</v>
       </c>
       <c r="K16" t="b">
         <v>0</v>
@@ -2658,7 +2656,7 @@
         <v>0</v>
       </c>
       <c r="M16" t="n">
-        <v>2222000</v>
+        <v>5000</v>
       </c>
       <c r="N16" t="n">
         <v>0</v>
@@ -2667,61 +2665,61 @@
         <v>0</v>
       </c>
       <c r="P16" t="n">
-        <v>220</v>
+        <v>150</v>
       </c>
       <c r="Q16" t="n">
-        <v>220</v>
+        <v>150</v>
       </c>
       <c r="R16" t="n">
-        <v>2275150</v>
+        <v>27000650</v>
       </c>
       <c r="S16" t="n">
-        <v>225.8</v>
+        <v>153.4</v>
       </c>
       <c r="T16" t="n">
-        <v>212.425</v>
+        <v>147.45</v>
       </c>
       <c r="U16" t="n">
-        <v>211.125</v>
+        <v>146.85</v>
       </c>
       <c r="V16" t="n">
-        <v>216.1166666666667</v>
+        <v>157.8916666666667</v>
       </c>
       <c r="W16" t="n">
-        <v>6.068834410018638</v>
+        <v>2.493686222751734</v>
       </c>
       <c r="X16" t="n">
-        <v>6.737541555554656</v>
+        <v>2.90857006187582</v>
       </c>
       <c r="Y16" t="n">
-        <v>-0.6687071455360174</v>
+        <v>-0.4148838391240863</v>
       </c>
       <c r="Z16" t="n">
-        <v>0.4393759495140168</v>
+        <v>0.1642919784818218</v>
       </c>
       <c r="AA16" t="b">
         <v>0</v>
       </c>
       <c r="AB16" t="n">
-        <v>0.134020618556701</v>
+        <v>0.08695652173913038</v>
       </c>
       <c r="AC16" t="n">
-        <v>-0.09278350515463918</v>
+        <v>-0.0625</v>
       </c>
       <c r="AD16" t="n">
-        <v>0.1258601385820362</v>
+        <v>0.07879604176446553</v>
       </c>
       <c r="AE16" t="n">
-        <v>-0.09948530168908409</v>
+        <v>-0.06920179653444491</v>
       </c>
       <c r="AF16" t="n">
-        <v>0.2253454402711202</v>
+        <v>0.1479978382989104</v>
       </c>
       <c r="AG16" t="n">
-        <v>88</v>
+        <v>80</v>
       </c>
       <c r="AH16" t="n">
-        <v>42</v>
+        <v>52</v>
       </c>
       <c r="AI16" t="b">
         <v>1</v>
@@ -2742,7 +2740,7 @@
         <v>1</v>
       </c>
       <c r="AO16" t="n">
-        <v>227.92</v>
+        <v>154.8</v>
       </c>
       <c r="AP16" t="inlineStr">
         <is>
@@ -2758,12 +2756,12 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>2481</t>
+          <t>6278</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>強茂</t>
+          <t>台表科</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -2772,7 +2770,7 @@
         </is>
       </c>
       <c r="E17" t="n">
-        <v>39.4</v>
+        <v>39</v>
       </c>
       <c r="F17" t="inlineStr">
         <is>
@@ -2781,15 +2779,15 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>20260911</t>
+          <t>20260914</t>
         </is>
       </c>
       <c r="H17" t="n">
-        <v>5000</v>
+        <v>3248000</v>
       </c>
       <c r="I17" t="inlineStr"/>
       <c r="J17" t="n">
-        <v>34</v>
+        <v>19</v>
       </c>
       <c r="K17" t="b">
         <v>0</v>
@@ -2798,7 +2796,7 @@
         <v>0</v>
       </c>
       <c r="M17" t="n">
-        <v>5000</v>
+        <v>3248000</v>
       </c>
       <c r="N17" t="n">
         <v>0</v>
@@ -2807,64 +2805,64 @@
         <v>0</v>
       </c>
       <c r="P17" t="n">
-        <v>150</v>
+        <v>186.5</v>
       </c>
       <c r="Q17" t="n">
-        <v>150</v>
+        <v>186.5</v>
       </c>
       <c r="R17" t="n">
-        <v>27240867</v>
+        <v>2109075</v>
       </c>
       <c r="S17" t="n">
-        <v>153.4</v>
+        <v>191</v>
       </c>
       <c r="T17" t="n">
-        <v>147.45</v>
+        <v>190.075</v>
       </c>
       <c r="U17" t="n">
-        <v>146.85</v>
+        <v>189.4</v>
       </c>
       <c r="V17" t="n">
-        <v>157.8916666666667</v>
+        <v>180.113899230957</v>
       </c>
       <c r="W17" t="n">
-        <v>2.493686222751734</v>
+        <v>2.21500964183187</v>
       </c>
       <c r="X17" t="n">
-        <v>2.90857006187582</v>
+        <v>4.819424623145751</v>
       </c>
       <c r="Y17" t="n">
-        <v>-0.4148838391240863</v>
+        <v>-2.604414981313881</v>
       </c>
       <c r="Z17" t="n">
-        <v>0.1642919784818218</v>
+        <v>-2.119228753447062</v>
       </c>
       <c r="AA17" t="b">
         <v>0</v>
       </c>
       <c r="AB17" t="n">
-        <v>0.08695652173913038</v>
+        <v>0.07803468208092479</v>
       </c>
       <c r="AC17" t="n">
-        <v>-0.0625</v>
+        <v>-0.06191761106456184</v>
       </c>
       <c r="AD17" t="n">
-        <v>0.07879604176446553</v>
+        <v>0.06987420210625994</v>
       </c>
       <c r="AE17" t="n">
-        <v>-0.06920179653444491</v>
+        <v>-0.06861940759900675</v>
       </c>
       <c r="AF17" t="n">
-        <v>0.1479978382989104</v>
+        <v>0.1384936097052667</v>
       </c>
       <c r="AG17" t="n">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="AH17" t="n">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="AI17" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AJ17" t="b">
         <v>1</v>
@@ -2882,7 +2880,7 @@
         <v>1</v>
       </c>
       <c r="AO17" t="n">
-        <v>154.8</v>
+        <v>215.97</v>
       </c>
       <c r="AP17" t="inlineStr">
         <is>
@@ -2898,12 +2896,12 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>6278</t>
+          <t>3037</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>台表科</t>
+          <t>欣興</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -2912,7 +2910,7 @@
         </is>
       </c>
       <c r="E18" t="n">
-        <v>39</v>
+        <v>37.8</v>
       </c>
       <c r="F18" t="inlineStr">
         <is>
@@ -2921,24 +2919,24 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>20260911</t>
+          <t>20260914</t>
         </is>
       </c>
       <c r="H18" t="n">
-        <v>3248000</v>
+        <v>20300000</v>
       </c>
       <c r="I18" t="inlineStr"/>
       <c r="J18" t="n">
-        <v>19</v>
+        <v>3</v>
       </c>
       <c r="K18" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L18" t="b">
         <v>0</v>
       </c>
       <c r="M18" t="n">
-        <v>3248000</v>
+        <v>20300000</v>
       </c>
       <c r="N18" t="n">
         <v>0</v>
@@ -2947,67 +2945,67 @@
         <v>0</v>
       </c>
       <c r="P18" t="n">
-        <v>186.5</v>
+        <v>977</v>
       </c>
       <c r="Q18" t="n">
-        <v>186.5</v>
+        <v>977</v>
       </c>
       <c r="R18" t="n">
-        <v>2168432</v>
+        <v>11021738</v>
       </c>
       <c r="S18" t="n">
-        <v>191</v>
+        <v>973.4</v>
       </c>
       <c r="T18" t="n">
-        <v>190.075</v>
+        <v>1043.75</v>
       </c>
       <c r="U18" t="n">
-        <v>189.4</v>
+        <v>1045.9</v>
       </c>
       <c r="V18" t="n">
-        <v>180.113899230957</v>
+        <v>954.378163655599</v>
       </c>
       <c r="W18" t="n">
-        <v>2.21500964183187</v>
+        <v>-15.22422037337219</v>
       </c>
       <c r="X18" t="n">
-        <v>4.819424623145729</v>
+        <v>-7.956888759828145</v>
       </c>
       <c r="Y18" t="n">
-        <v>-2.604414981313859</v>
+        <v>-7.267331613544046</v>
       </c>
       <c r="Z18" t="n">
-        <v>-2.119228753447034</v>
+        <v>-10.2807709018258</v>
       </c>
       <c r="AA18" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AB18" t="n">
-        <v>0.07803468208092479</v>
+        <v>-0.042156862745098</v>
       </c>
       <c r="AC18" t="n">
-        <v>-0.06191761106456184</v>
+        <v>0.01136422295068207</v>
       </c>
       <c r="AD18" t="n">
-        <v>0.06987420210625994</v>
+        <v>-0.05031734271976285</v>
       </c>
       <c r="AE18" t="n">
-        <v>-0.06861940759900675</v>
+        <v>0.004662426416237153</v>
       </c>
       <c r="AF18" t="n">
-        <v>0.1384936097052667</v>
+        <v>-0.054979769136</v>
       </c>
       <c r="AG18" t="n">
-        <v>78</v>
+        <v>34</v>
       </c>
       <c r="AH18" t="n">
-        <v>54</v>
+        <v>74</v>
       </c>
       <c r="AI18" t="b">
         <v>0</v>
       </c>
       <c r="AJ18" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AK18" t="b">
         <v>0</v>
@@ -3016,18 +3014,16 @@
         <v>0</v>
       </c>
       <c r="AM18" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AN18" t="b">
         <v>1</v>
       </c>
       <c r="AO18" t="n">
-        <v>215.97</v>
-      </c>
-      <c r="AP18" t="inlineStr">
-        <is>
-          <t>Already Up</t>
-        </is>
+        <v>1059.07</v>
+      </c>
+      <c r="AP18" t="n">
+        <v>1190.26</v>
       </c>
     </row>
     <row r="19">
@@ -3038,12 +3034,12 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>3037</t>
+          <t>3264</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>欣興</t>
+          <t>欣銓</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -3052,7 +3048,7 @@
         </is>
       </c>
       <c r="E19" t="n">
-        <v>37.8</v>
+        <v>36.6</v>
       </c>
       <c r="F19" t="inlineStr">
         <is>
@@ -3061,24 +3057,24 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>20260911</t>
+          <t>20260914</t>
         </is>
       </c>
       <c r="H19" t="n">
-        <v>20300000</v>
+        <v>5028000</v>
       </c>
       <c r="I19" t="inlineStr"/>
       <c r="J19" t="n">
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="K19" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L19" t="b">
         <v>0</v>
       </c>
       <c r="M19" t="n">
-        <v>20300000</v>
+        <v>5028000</v>
       </c>
       <c r="N19" t="n">
         <v>0</v>
@@ -3087,85 +3083,89 @@
         <v>0</v>
       </c>
       <c r="P19" t="n">
-        <v>977</v>
+        <v>230.5</v>
       </c>
       <c r="Q19" t="n">
-        <v>977</v>
+        <v>230.5</v>
       </c>
       <c r="R19" t="n">
-        <v>11402888</v>
+        <v>6490514</v>
       </c>
       <c r="S19" t="n">
-        <v>973.4</v>
+        <v>231.1</v>
       </c>
       <c r="T19" t="n">
-        <v>1043.75</v>
+        <v>222.275</v>
       </c>
       <c r="U19" t="n">
-        <v>1045.9</v>
+        <v>222.025</v>
       </c>
       <c r="V19" t="n">
-        <v>954.378163655599</v>
+        <v>218.5139709472656</v>
       </c>
       <c r="W19" t="n">
-        <v>-15.22422037337219</v>
+        <v>4.54476695639687</v>
       </c>
       <c r="X19" t="n">
-        <v>-7.956888759828141</v>
+        <v>4.419014901357135</v>
       </c>
       <c r="Y19" t="n">
-        <v>-7.26733161354405</v>
+        <v>0.1257520550397349</v>
       </c>
       <c r="Z19" t="n">
-        <v>-10.28077090182581</v>
+        <v>0.7171665199265824</v>
       </c>
       <c r="AA19" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AB19" t="n">
-        <v>-0.042156862745098</v>
+        <v>0.02217294900221733</v>
       </c>
       <c r="AC19" t="n">
-        <v>0.01136422295068207</v>
+        <v>0.01110383392943382</v>
       </c>
       <c r="AD19" t="n">
-        <v>-0.05031734271976285</v>
+        <v>0.01401246902755249</v>
       </c>
       <c r="AE19" t="n">
-        <v>0.004662426416237153</v>
+        <v>0.0044020373949889</v>
       </c>
       <c r="AF19" t="n">
-        <v>-0.054979769136</v>
+        <v>0.009610431632563587</v>
       </c>
       <c r="AG19" t="n">
-        <v>34</v>
+        <v>64</v>
       </c>
       <c r="AH19" t="n">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="AI19" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AJ19" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AK19" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AL19" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AM19" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AN19" t="b">
-        <v>1</v>
-      </c>
-      <c r="AO19" t="n">
-        <v>1059.07</v>
-      </c>
-      <c r="AP19" t="n">
-        <v>1190.26</v>
+        <v>0</v>
+      </c>
+      <c r="AO19" t="inlineStr">
+        <is>
+          <t>Already &gt; 0</t>
+        </is>
+      </c>
+      <c r="AP19" t="inlineStr">
+        <is>
+          <t>Already Up</t>
+        </is>
       </c>
     </row>
     <row r="20">
@@ -3176,12 +3176,12 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>3264</t>
+          <t>8358</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>欣銓</t>
+          <t>金居</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -3199,15 +3199,15 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>20260911</t>
+          <t>20260914</t>
         </is>
       </c>
       <c r="H20" t="n">
-        <v>5028000</v>
+        <v>1000</v>
       </c>
       <c r="I20" t="inlineStr"/>
       <c r="J20" t="n">
-        <v>15</v>
+        <v>50</v>
       </c>
       <c r="K20" t="b">
         <v>0</v>
@@ -3216,7 +3216,7 @@
         <v>0</v>
       </c>
       <c r="M20" t="n">
-        <v>5028000</v>
+        <v>1000</v>
       </c>
       <c r="N20" t="n">
         <v>0</v>
@@ -3225,61 +3225,61 @@
         <v>0</v>
       </c>
       <c r="P20" t="n">
-        <v>230.5</v>
+        <v>485</v>
       </c>
       <c r="Q20" t="n">
-        <v>230.5</v>
+        <v>485</v>
       </c>
       <c r="R20" t="n">
-        <v>6599333</v>
+        <v>13838378</v>
       </c>
       <c r="S20" t="n">
-        <v>231.1</v>
+        <v>513.4</v>
       </c>
       <c r="T20" t="n">
-        <v>222.275</v>
+        <v>476.7</v>
       </c>
       <c r="U20" t="n">
-        <v>222.025</v>
+        <v>473.875</v>
       </c>
       <c r="V20" t="n">
-        <v>218.5139709472656</v>
+        <v>462.8774480183919</v>
       </c>
       <c r="W20" t="n">
-        <v>4.54476695639687</v>
+        <v>18.27184947733946</v>
       </c>
       <c r="X20" t="n">
-        <v>4.419014901357135</v>
+        <v>23.08834182168413</v>
       </c>
       <c r="Y20" t="n">
-        <v>0.1257520550397349</v>
+        <v>-4.816492344344674</v>
       </c>
       <c r="Z20" t="n">
-        <v>0.7171665199265824</v>
+        <v>-0.6158480075517936</v>
       </c>
       <c r="AA20" t="b">
         <v>0</v>
       </c>
       <c r="AB20" t="n">
-        <v>0.02217294900221733</v>
+        <v>0.1318553092182031</v>
       </c>
       <c r="AC20" t="n">
-        <v>0.01110383392943382</v>
+        <v>-0.3039718654059238</v>
       </c>
       <c r="AD20" t="n">
-        <v>0.01401246902755249</v>
+        <v>0.1236948292435383</v>
       </c>
       <c r="AE20" t="n">
-        <v>0.0044020373949889</v>
+        <v>-0.3106736619403687</v>
       </c>
       <c r="AF20" t="n">
-        <v>0.009610431632563587</v>
+        <v>0.434368491183907</v>
       </c>
       <c r="AG20" t="n">
-        <v>64</v>
+        <v>86</v>
       </c>
       <c r="AH20" t="n">
-        <v>72</v>
+        <v>6</v>
       </c>
       <c r="AI20" t="b">
         <v>1</v>
@@ -3288,21 +3288,19 @@
         <v>1</v>
       </c>
       <c r="AK20" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AL20" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AM20" t="b">
         <v>0</v>
       </c>
       <c r="AN20" t="b">
-        <v>0</v>
-      </c>
-      <c r="AO20" t="inlineStr">
-        <is>
-          <t>Already &gt; 0</t>
-        </is>
+        <v>1</v>
+      </c>
+      <c r="AO20" t="n">
+        <v>539.3200000000001</v>
       </c>
       <c r="AP20" t="inlineStr">
         <is>
@@ -3318,12 +3316,12 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>8358</t>
+          <t>2382</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>金居</t>
+          <t>廣達</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -3332,7 +3330,7 @@
         </is>
       </c>
       <c r="E21" t="n">
-        <v>36.6</v>
+        <v>34.8</v>
       </c>
       <c r="F21" t="inlineStr">
         <is>
@@ -3341,7 +3339,7 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>20260911</t>
+          <t>20260914</t>
         </is>
       </c>
       <c r="H21" t="n">
@@ -3349,7 +3347,7 @@
       </c>
       <c r="I21" t="inlineStr"/>
       <c r="J21" t="n">
-        <v>50</v>
+        <v>37</v>
       </c>
       <c r="K21" t="b">
         <v>0</v>
@@ -3367,61 +3365,61 @@
         <v>0</v>
       </c>
       <c r="P21" t="n">
-        <v>485</v>
+        <v>336.5</v>
       </c>
       <c r="Q21" t="n">
-        <v>485</v>
+        <v>336.5</v>
       </c>
       <c r="R21" t="n">
-        <v>14656857</v>
+        <v>10850704</v>
       </c>
       <c r="S21" t="n">
-        <v>513.4</v>
+        <v>338</v>
       </c>
       <c r="T21" t="n">
-        <v>476.7</v>
+        <v>333.975</v>
       </c>
       <c r="U21" t="n">
-        <v>473.875</v>
+        <v>333.525</v>
       </c>
       <c r="V21" t="n">
-        <v>462.8774480183919</v>
+        <v>334.3058400472005</v>
       </c>
       <c r="W21" t="n">
-        <v>18.27184947733946</v>
+        <v>2.73096366220733</v>
       </c>
       <c r="X21" t="n">
-        <v>23.08834182168414</v>
+        <v>3.584727047892501</v>
       </c>
       <c r="Y21" t="n">
-        <v>-4.816492344344681</v>
+        <v>-0.8537633856851707</v>
       </c>
       <c r="Z21" t="n">
-        <v>-0.6158480075518042</v>
+        <v>-0.6029421409144229</v>
       </c>
       <c r="AA21" t="b">
         <v>0</v>
       </c>
       <c r="AB21" t="n">
-        <v>0.1318553092182031</v>
+        <v>0.02748091603053426</v>
       </c>
       <c r="AC21" t="n">
-        <v>-0.3039718654059238</v>
+        <v>-0.06684531260895965</v>
       </c>
       <c r="AD21" t="n">
-        <v>0.1236948292435383</v>
+        <v>0.01932043605586942</v>
       </c>
       <c r="AE21" t="n">
-        <v>-0.3106736619403687</v>
+        <v>-0.07354710914340457</v>
       </c>
       <c r="AF21" t="n">
-        <v>0.434368491183907</v>
+        <v>0.09286754519927398</v>
       </c>
       <c r="AG21" t="n">
-        <v>86</v>
+        <v>66</v>
       </c>
       <c r="AH21" t="n">
-        <v>6</v>
+        <v>48</v>
       </c>
       <c r="AI21" t="b">
         <v>1</v>
@@ -3442,7 +3440,7 @@
         <v>1</v>
       </c>
       <c r="AO21" t="n">
-        <v>539.3200000000001</v>
+        <v>346.6</v>
       </c>
       <c r="AP21" t="inlineStr">
         <is>
@@ -3458,12 +3456,12 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>2382</t>
+          <t>6510</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>廣達</t>
+          <t>精測</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -3476,20 +3474,20 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Heavy Sell</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>20260911</t>
+          <t>20260914</t>
         </is>
       </c>
       <c r="H22" t="n">
-        <v>1000</v>
+        <v>446000</v>
       </c>
       <c r="I22" t="inlineStr"/>
       <c r="J22" t="n">
-        <v>37</v>
+        <v>29</v>
       </c>
       <c r="K22" t="b">
         <v>0</v>
@@ -3498,70 +3496,70 @@
         <v>0</v>
       </c>
       <c r="M22" t="n">
-        <v>1000</v>
+        <v>637000</v>
       </c>
       <c r="N22" t="n">
-        <v>0</v>
+        <v>-191000</v>
       </c>
       <c r="O22" t="n">
-        <v>0</v>
+        <v>-0.2998430141287284</v>
       </c>
       <c r="P22" t="n">
-        <v>336.5</v>
+        <v>3480</v>
       </c>
       <c r="Q22" t="n">
-        <v>336.5</v>
+        <v>3480</v>
       </c>
       <c r="R22" t="n">
-        <v>10997504</v>
+        <v>1060301</v>
       </c>
       <c r="S22" t="n">
-        <v>338</v>
+        <v>3570</v>
       </c>
       <c r="T22" t="n">
-        <v>333.975</v>
+        <v>3052</v>
       </c>
       <c r="U22" t="n">
-        <v>333.525</v>
+        <v>3027.5</v>
       </c>
       <c r="V22" t="n">
-        <v>334.3058400472005</v>
+        <v>2927.079142252604</v>
       </c>
       <c r="W22" t="n">
-        <v>2.73096366220733</v>
+        <v>210.4160916274086</v>
       </c>
       <c r="X22" t="n">
-        <v>3.584727047892501</v>
+        <v>165.3148866757759</v>
       </c>
       <c r="Y22" t="n">
-        <v>-0.8537633856851707</v>
+        <v>45.10120495163272</v>
       </c>
       <c r="Z22" t="n">
-        <v>-0.6029421409144229</v>
+        <v>76.13910869752348</v>
       </c>
       <c r="AA22" t="b">
         <v>0</v>
       </c>
       <c r="AB22" t="n">
-        <v>0.02748091603053426</v>
+        <v>0.1638795986622072</v>
       </c>
       <c r="AC22" t="n">
-        <v>-0.06684531260895965</v>
+        <v>-0.03081196953418652</v>
       </c>
       <c r="AD22" t="n">
-        <v>0.01932043605586942</v>
+        <v>0.1557191186875424</v>
       </c>
       <c r="AE22" t="n">
-        <v>-0.07354710914340457</v>
+        <v>-0.03751376606863144</v>
       </c>
       <c r="AF22" t="n">
-        <v>0.09286754519927398</v>
+        <v>0.1932328847561738</v>
       </c>
       <c r="AG22" t="n">
-        <v>66</v>
+        <v>92</v>
       </c>
       <c r="AH22" t="n">
-        <v>48</v>
+        <v>64</v>
       </c>
       <c r="AI22" t="b">
         <v>1</v>
@@ -3570,19 +3568,21 @@
         <v>1</v>
       </c>
       <c r="AK22" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AL22" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AM22" t="b">
         <v>0</v>
       </c>
       <c r="AN22" t="b">
-        <v>1</v>
-      </c>
-      <c r="AO22" t="n">
-        <v>346.6</v>
+        <v>0</v>
+      </c>
+      <c r="AO22" t="inlineStr">
+        <is>
+          <t>Already &gt; 0</t>
+        </is>
       </c>
       <c r="AP22" t="inlineStr">
         <is>
@@ -3621,7 +3621,7 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>20260911</t>
+          <t>20260914</t>
         </is>
       </c>
       <c r="H23" t="n">
@@ -3653,7 +3653,7 @@
         <v>17885</v>
       </c>
       <c r="R23" t="n">
-        <v>229307</v>
+        <v>206906</v>
       </c>
       <c r="S23" t="n">
         <v>18725</v>
@@ -3763,7 +3763,7 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>20260911</t>
+          <t>20260914</t>
         </is>
       </c>
       <c r="H24" t="n">
@@ -3795,7 +3795,7 @@
         <v>531</v>
       </c>
       <c r="R24" t="n">
-        <v>1934780</v>
+        <v>1776618</v>
       </c>
       <c r="S24" t="n">
         <v>581.4</v>
@@ -3813,13 +3813,13 @@
         <v>4.542231291026837</v>
       </c>
       <c r="X24" t="n">
-        <v>18.69904312455205</v>
+        <v>18.69904312455204</v>
       </c>
       <c r="Y24" t="n">
         <v>-14.15681183352521</v>
       </c>
       <c r="Z24" t="n">
-        <v>-9.085081964823583</v>
+        <v>-9.085081964823576</v>
       </c>
       <c r="AA24" t="b">
         <v>0</v>
@@ -3901,7 +3901,7 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>20260911</t>
+          <t>20260914</t>
         </is>
       </c>
       <c r="H25" t="n">
@@ -3909,7 +3909,7 @@
       </c>
       <c r="I25" t="inlineStr"/>
       <c r="J25" t="n">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="K25" t="b">
         <v>0</v>
@@ -3933,7 +3933,7 @@
         <v>221.5</v>
       </c>
       <c r="R25" t="n">
-        <v>9309091</v>
+        <v>8951713</v>
       </c>
       <c r="S25" t="n">
         <v>229.2</v>
@@ -4039,7 +4039,7 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>20260911</t>
+          <t>20260914</t>
         </is>
       </c>
       <c r="H26" t="n">
@@ -4071,7 +4071,7 @@
         <v>1080</v>
       </c>
       <c r="R26" t="n">
-        <v>6332246</v>
+        <v>6190632</v>
       </c>
       <c r="S26" t="n">
         <v>1067</v>
@@ -4089,13 +4089,13 @@
         <v>-28.25392534665025</v>
       </c>
       <c r="X26" t="n">
-        <v>-15.05066810371136</v>
+        <v>-15.05066810371143</v>
       </c>
       <c r="Y26" t="n">
-        <v>-13.20325724293889</v>
+        <v>-13.20325724293882</v>
       </c>
       <c r="Z26" t="n">
-        <v>-17.55514346907307</v>
+        <v>-17.55514346907299</v>
       </c>
       <c r="AA26" t="b">
         <v>1</v>
@@ -4177,7 +4177,7 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>20260911</t>
+          <t>20260914</t>
         </is>
       </c>
       <c r="H27" t="n">
@@ -4209,7 +4209,7 @@
         <v>18.89999961853027</v>
       </c>
       <c r="R27" t="n">
-        <v>26774343</v>
+        <v>26719960</v>
       </c>
       <c r="S27" t="n">
         <v>19.07000007629394</v>
@@ -4227,13 +4227,13 @@
         <v>-0.02029280309746895</v>
       </c>
       <c r="X27" t="n">
-        <v>-0.004584705488016895</v>
+        <v>-0.00458470548801689</v>
       </c>
       <c r="Y27" t="n">
-        <v>-0.01570809760945205</v>
+        <v>-0.01570809760945206</v>
       </c>
       <c r="Z27" t="n">
-        <v>0.003710652179192185</v>
+        <v>0.003710652179192178</v>
       </c>
       <c r="AA27" t="b">
         <v>0</v>
@@ -4315,7 +4315,7 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>20260911</t>
+          <t>20260914</t>
         </is>
       </c>
       <c r="H28" t="n">
@@ -4347,7 +4347,7 @@
         <v>1250</v>
       </c>
       <c r="R28" t="n">
-        <v>1654954</v>
+        <v>1568860</v>
       </c>
       <c r="S28" t="n">
         <v>1323</v>
@@ -4451,7 +4451,7 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>20260911</t>
+          <t>20260914</t>
         </is>
       </c>
       <c r="H29" t="n">
@@ -4483,7 +4483,7 @@
         <v>493</v>
       </c>
       <c r="R29" t="n">
-        <v>38361401</v>
+        <v>36289746</v>
       </c>
       <c r="S29" t="n">
         <v>515.8</v>
@@ -4498,16 +4498,16 @@
         <v>461.0137659708659</v>
       </c>
       <c r="W29" t="n">
-        <v>3.08743414741798</v>
+        <v>3.087434147418037</v>
       </c>
       <c r="X29" t="n">
-        <v>8.592254632288753</v>
+        <v>8.592254632288817</v>
       </c>
       <c r="Y29" t="n">
-        <v>-5.504820484870773</v>
+        <v>-5.50482048487078</v>
       </c>
       <c r="Z29" t="n">
-        <v>-3.555447643126836</v>
+        <v>-3.555447643126843</v>
       </c>
       <c r="AA29" t="b">
         <v>0</v>
@@ -4589,7 +4589,7 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>20260911</t>
+          <t>20260914</t>
         </is>
       </c>
       <c r="H30" t="n">
@@ -4621,7 +4621,7 @@
         <v>6890</v>
       </c>
       <c r="R30" t="n">
-        <v>477442</v>
+        <v>439537</v>
       </c>
       <c r="S30" t="n">
         <v>7213</v>
@@ -4731,7 +4731,7 @@
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>20260911</t>
+          <t>20260914</t>
         </is>
       </c>
       <c r="H31" t="n">
@@ -4763,7 +4763,7 @@
         <v>1030</v>
       </c>
       <c r="R31" t="n">
-        <v>4392806</v>
+        <v>4200828</v>
       </c>
       <c r="S31" t="n">
         <v>1074</v>
@@ -4871,7 +4871,7 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>20260911</t>
+          <t>20260914</t>
         </is>
       </c>
       <c r="H32" t="n">
@@ -4903,7 +4903,7 @@
         <v>495</v>
       </c>
       <c r="R32" t="n">
-        <v>18704156</v>
+        <v>18333613</v>
       </c>
       <c r="S32" t="n">
         <v>499.5</v>
@@ -5013,7 +5013,7 @@
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>20260911</t>
+          <t>20260914</t>
         </is>
       </c>
       <c r="H33" t="n">
@@ -5045,7 +5045,7 @@
         <v>76.5</v>
       </c>
       <c r="R33" t="n">
-        <v>742720</v>
+        <v>730131</v>
       </c>
       <c r="S33" t="n">
         <v>76.31999969482422</v>
@@ -5063,13 +5063,13 @@
         <v>-0.3923867331361492</v>
       </c>
       <c r="X33" t="n">
-        <v>-0.2160973872349223</v>
+        <v>-0.2160973872349232</v>
       </c>
       <c r="Y33" t="n">
-        <v>-0.176289345901227</v>
+        <v>-0.1762893459012261</v>
       </c>
       <c r="Z33" t="n">
-        <v>-0.2149443420343282</v>
+        <v>-0.2149443420343271</v>
       </c>
       <c r="AA33" t="b">
         <v>1</v>
@@ -5151,7 +5151,7 @@
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>20260911</t>
+          <t>20260914</t>
         </is>
       </c>
       <c r="H34" t="n">
@@ -5183,7 +5183,7 @@
         <v>157.5</v>
       </c>
       <c r="R34" t="n">
-        <v>8916668</v>
+        <v>8835730</v>
       </c>
       <c r="S34" t="n">
         <v>156.8</v>
@@ -5201,13 +5201,13 @@
         <v>1.022531623645705</v>
       </c>
       <c r="X34" t="n">
-        <v>-0.3608630683825204</v>
+        <v>-0.3608630683825206</v>
       </c>
       <c r="Y34" t="n">
         <v>1.383394692028225</v>
       </c>
       <c r="Z34" t="n">
-        <v>1.531623059900007</v>
+        <v>1.531623059900008</v>
       </c>
       <c r="AA34" t="b">
         <v>0</v>
@@ -5291,7 +5291,7 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>20260911</t>
+          <t>20260914</t>
         </is>
       </c>
       <c r="H35" t="n">
@@ -5323,7 +5323,7 @@
         <v>183</v>
       </c>
       <c r="R35" t="n">
-        <v>6099711</v>
+        <v>5939599</v>
       </c>
       <c r="S35" t="n">
         <v>197.7</v>
@@ -5338,16 +5338,16 @@
         <v>190.8137947082519</v>
       </c>
       <c r="W35" t="n">
-        <v>-0.5061848703785756</v>
+        <v>-0.5061848703786325</v>
       </c>
       <c r="X35" t="n">
-        <v>3.391017077474064</v>
+        <v>3.391017077474009</v>
       </c>
       <c r="Y35" t="n">
-        <v>-3.89720194785264</v>
+        <v>-3.897201947852642</v>
       </c>
       <c r="Z35" t="n">
-        <v>-2.538479135708376</v>
+        <v>-2.538479135708378</v>
       </c>
       <c r="AA35" t="b">
         <v>0</v>
@@ -5427,7 +5427,7 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>20260911</t>
+          <t>20260914</t>
         </is>
       </c>
       <c r="H36" t="n">
@@ -5459,7 +5459,7 @@
         <v>544</v>
       </c>
       <c r="R36" t="n">
-        <v>35425208</v>
+        <v>33780557</v>
       </c>
       <c r="S36" t="n">
         <v>567.4</v>
@@ -5567,7 +5567,7 @@
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>20260911</t>
+          <t>20260914</t>
         </is>
       </c>
       <c r="H37" t="n">
@@ -5599,7 +5599,7 @@
         <v>248</v>
       </c>
       <c r="R37" t="n">
-        <v>24087118</v>
+        <v>23496234</v>
       </c>
       <c r="S37" t="n">
         <v>251.7</v>
@@ -5617,13 +5617,13 @@
         <v>-0.194215886037</v>
       </c>
       <c r="X37" t="n">
-        <v>0.09963341641249436</v>
+        <v>0.09963341641249028</v>
       </c>
       <c r="Y37" t="n">
-        <v>-0.2938493024494944</v>
+        <v>-0.2938493024494903</v>
       </c>
       <c r="Z37" t="n">
-        <v>0.103580516305714</v>
+        <v>0.1035805163057191</v>
       </c>
       <c r="AA37" t="b">
         <v>0</v>
@@ -5705,7 +5705,7 @@
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>20260911</t>
+          <t>20260914</t>
         </is>
       </c>
       <c r="H38" t="n">
@@ -5737,7 +5737,7 @@
         <v>1620</v>
       </c>
       <c r="R38" t="n">
-        <v>15864605</v>
+        <v>13791960</v>
       </c>
       <c r="S38" t="n">
         <v>1749</v>
@@ -5755,13 +5755,13 @@
         <v>-22.02418909344351</v>
       </c>
       <c r="X38" t="n">
-        <v>0.5316347932180951</v>
+        <v>0.5316347932180774</v>
       </c>
       <c r="Y38" t="n">
-        <v>-22.55582388666161</v>
+        <v>-22.55582388666159</v>
       </c>
       <c r="Z38" t="n">
-        <v>-11.6528857795805</v>
+        <v>-11.65288577958048</v>
       </c>
       <c r="AA38" t="b">
         <v>0</v>
@@ -5843,7 +5843,7 @@
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>20260911</t>
+          <t>20260914</t>
         </is>
       </c>
       <c r="H39" t="n">
@@ -5875,7 +5875,7 @@
         <v>82.30000305175781</v>
       </c>
       <c r="R39" t="n">
-        <v>979637</v>
+        <v>962201</v>
       </c>
       <c r="S39" t="n">
         <v>82.38000030517578</v>
@@ -5893,13 +5893,13 @@
         <v>-0.5113076913983434</v>
       </c>
       <c r="X39" t="n">
-        <v>-0.6317935496088432</v>
+        <v>-0.6317935496088464</v>
       </c>
       <c r="Y39" t="n">
-        <v>0.1204858582104997</v>
+        <v>0.1204858582105029</v>
       </c>
       <c r="Z39" t="n">
-        <v>0.1203361515534197</v>
+        <v>0.1203361515534237</v>
       </c>
       <c r="AA39" t="b">
         <v>1</v>
@@ -5983,7 +5983,7 @@
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>20260911</t>
+          <t>20260914</t>
         </is>
       </c>
       <c r="H40" t="n">
@@ -6015,7 +6015,7 @@
         <v>1885</v>
       </c>
       <c r="R40" t="n">
-        <v>3754695</v>
+        <v>3345431</v>
       </c>
       <c r="S40" t="n">
         <v>1984</v>
@@ -6033,13 +6033,13 @@
         <v>-55.49182145008945</v>
       </c>
       <c r="X40" t="n">
-        <v>-36.5421283528112</v>
+        <v>-36.54212835281149</v>
       </c>
       <c r="Y40" t="n">
-        <v>-18.94969309727825</v>
+        <v>-18.94969309727796</v>
       </c>
       <c r="Z40" t="n">
-        <v>-11.28142977941302</v>
+        <v>-11.28142977941265</v>
       </c>
       <c r="AA40" t="b">
         <v>0</v>
@@ -6121,7 +6121,7 @@
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>20260911</t>
+          <t>20260914</t>
         </is>
       </c>
       <c r="H41" t="n">
@@ -6153,7 +6153,7 @@
         <v>2160</v>
       </c>
       <c r="R41" t="n">
-        <v>2244731</v>
+        <v>2196224</v>
       </c>
       <c r="S41" t="n">
         <v>2234</v>
@@ -6261,7 +6261,7 @@
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>20260911</t>
+          <t>20260914</t>
         </is>
       </c>
       <c r="H42" t="n">
@@ -6293,7 +6293,7 @@
         <v>86.69999694824219</v>
       </c>
       <c r="R42" t="n">
-        <v>22151183</v>
+        <v>21780838</v>
       </c>
       <c r="S42" t="n">
         <v>90.14000091552734</v>
@@ -6311,13 +6311,13 @@
         <v>-0.1504473050209327</v>
       </c>
       <c r="X42" t="n">
-        <v>0.06893441592339129</v>
+        <v>0.06893441592339755</v>
       </c>
       <c r="Y42" t="n">
-        <v>-0.219381720944324</v>
+        <v>-0.2193817209443303</v>
       </c>
       <c r="Z42" t="n">
-        <v>0.1996662006369617</v>
+        <v>0.1996662006369538</v>
       </c>
       <c r="AA42" t="b">
         <v>0</v>
@@ -6399,7 +6399,7 @@
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>20260911</t>
+          <t>20260914</t>
         </is>
       </c>
       <c r="H43" t="n">
@@ -6431,7 +6431,7 @@
         <v>1285</v>
       </c>
       <c r="R43" t="n">
-        <v>1172895</v>
+        <v>1155113</v>
       </c>
       <c r="S43" t="n">
         <v>1325</v>
@@ -6446,16 +6446,16 @@
         <v>1390.675382486979</v>
       </c>
       <c r="W43" t="n">
-        <v>-38.34298079699261</v>
+        <v>-38.34298079699283</v>
       </c>
       <c r="X43" t="n">
-        <v>-22.40858140587961</v>
+        <v>-22.40858140587989</v>
       </c>
       <c r="Y43" t="n">
-        <v>-15.934399391113</v>
+        <v>-15.93439939111294</v>
       </c>
       <c r="Z43" t="n">
-        <v>-15.25202152236529</v>
+        <v>-15.25202152236522</v>
       </c>
       <c r="AA43" t="b">
         <v>0</v>
@@ -6537,7 +6537,7 @@
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>20260911</t>
+          <t>20260914</t>
         </is>
       </c>
       <c r="H44" t="n">
@@ -6569,7 +6569,7 @@
         <v>5365</v>
       </c>
       <c r="R44" t="n">
-        <v>1091759</v>
+        <v>1026967</v>
       </c>
       <c r="S44" t="n">
         <v>5390</v>
@@ -6587,13 +6587,13 @@
         <v>-46.36179370292848</v>
       </c>
       <c r="X44" t="n">
-        <v>-12.48951245917342</v>
+        <v>-12.48951245917341</v>
       </c>
       <c r="Y44" t="n">
-        <v>-33.87228124375506</v>
+        <v>-33.87228124375507</v>
       </c>
       <c r="Z44" t="n">
-        <v>-40.73263141229518</v>
+        <v>-40.73263141229519</v>
       </c>
       <c r="AA44" t="b">
         <v>1</v>
@@ -6675,7 +6675,7 @@
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>20260911</t>
+          <t>20260914</t>
         </is>
       </c>
       <c r="H45" t="n">
@@ -6707,7 +6707,7 @@
         <v>528</v>
       </c>
       <c r="R45" t="n">
-        <v>339481</v>
+        <v>304420</v>
       </c>
       <c r="S45" t="n">
         <v>546.2</v>
@@ -6725,13 +6725,13 @@
         <v>-9.930945072670511</v>
       </c>
       <c r="X45" t="n">
-        <v>-5.218066277923405</v>
+        <v>-5.218066277923453</v>
       </c>
       <c r="Y45" t="n">
-        <v>-4.712878794747106</v>
+        <v>-4.712878794747057</v>
       </c>
       <c r="Z45" t="n">
-        <v>-3.500110160440482</v>
+        <v>-3.50011016044042</v>
       </c>
       <c r="AA45" t="b">
         <v>0</v>
@@ -6813,7 +6813,7 @@
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>20260911</t>
+          <t>20260914</t>
         </is>
       </c>
       <c r="H46" t="n">
@@ -6845,7 +6845,7 @@
         <v>902</v>
       </c>
       <c r="R46" t="n">
-        <v>4732383</v>
+        <v>4384025</v>
       </c>
       <c r="S46" t="n">
         <v>940</v>
@@ -6860,16 +6860,16 @@
         <v>1047.686532592773</v>
       </c>
       <c r="W46" t="n">
-        <v>-13.5536782224533</v>
+        <v>-13.55367822245341</v>
       </c>
       <c r="X46" t="n">
-        <v>-8.069000559767273</v>
+        <v>-8.069000559767488</v>
       </c>
       <c r="Y46" t="n">
-        <v>-5.484677662686027</v>
+        <v>-5.484677662685925</v>
       </c>
       <c r="Z46" t="n">
-        <v>-2.415558947232716</v>
+        <v>-2.41555894723259</v>
       </c>
       <c r="AA46" t="b">
         <v>0</v>
@@ -6951,7 +6951,7 @@
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>20260911</t>
+          <t>20260914</t>
         </is>
       </c>
       <c r="H47" t="n">
@@ -6983,7 +6983,7 @@
         <v>900</v>
       </c>
       <c r="R47" t="n">
-        <v>748149</v>
+        <v>662890</v>
       </c>
       <c r="S47" t="n">
         <v>914</v>
@@ -7089,7 +7089,7 @@
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>20260911</t>
+          <t>20260914</t>
         </is>
       </c>
       <c r="H48" t="n">
@@ -7121,7 +7121,7 @@
         <v>5620</v>
       </c>
       <c r="R48" t="n">
-        <v>737868</v>
+        <v>682671</v>
       </c>
       <c r="S48" t="n">
         <v>5628</v>
@@ -7229,7 +7229,7 @@
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>20260911</t>
+          <t>20260914</t>
         </is>
       </c>
       <c r="H49" t="n">
@@ -7261,7 +7261,7 @@
         <v>3650</v>
       </c>
       <c r="R49" t="n">
-        <v>5577395</v>
+        <v>4843755</v>
       </c>
       <c r="S49" t="n">
         <v>3936</v>
@@ -7276,16 +7276,16 @@
         <v>3842.62412516276</v>
       </c>
       <c r="W49" t="n">
-        <v>8.454417129689773</v>
+        <v>8.454417129688409</v>
       </c>
       <c r="X49" t="n">
-        <v>65.33279409402078</v>
+        <v>65.33279409401921</v>
       </c>
       <c r="Y49" t="n">
-        <v>-56.87837696433101</v>
+        <v>-56.8783769643308</v>
       </c>
       <c r="Z49" t="n">
-        <v>-22.6162914770495</v>
+        <v>-22.61629147704922</v>
       </c>
       <c r="AA49" t="b">
         <v>0</v>
@@ -7367,7 +7367,7 @@
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>20260911</t>
+          <t>20260914</t>
         </is>
       </c>
       <c r="H50" t="n">
@@ -7399,7 +7399,7 @@
         <v>1875</v>
       </c>
       <c r="R50" t="n">
-        <v>1894326</v>
+        <v>1729263</v>
       </c>
       <c r="S50" t="n">
         <v>1957</v>
@@ -7503,7 +7503,7 @@
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>20260911</t>
+          <t>20260914</t>
         </is>
       </c>
       <c r="H51" t="n">
@@ -7535,7 +7535,7 @@
         <v>1365</v>
       </c>
       <c r="R51" t="n">
-        <v>4601278</v>
+        <v>4438145</v>
       </c>
       <c r="S51" t="n">
         <v>1364</v>
@@ -7553,10 +7553,10 @@
         <v>-28.33139062945816</v>
       </c>
       <c r="X51" t="n">
-        <v>-20.39418930163114</v>
+        <v>-20.39418930163115</v>
       </c>
       <c r="Y51" t="n">
-        <v>-7.937201327827012</v>
+        <v>-7.937201327827005</v>
       </c>
       <c r="Z51" t="n">
         <v>-10.82961256345573</v>

</xml_diff>